<commit_message>
chore: actualizar concentrados de capturas y remplazados
</commit_message>
<xml_diff>
--- a/salidas/CONSOLIDADO.xlsx
+++ b/salidas/CONSOLIDADO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,45 +454,70 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>correo_electronico</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>foto_1_path</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>foto_2_path</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>foto_1_kb</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>foto_2_kb</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>calle</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>numero</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>manzana_inegi</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>manzana</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>lote</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>curp</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>coordenadas_gps</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>direccion_base</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>fecha_captura</t>
         </is>
@@ -534,39 +559,44 @@
           <t>5555555555</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>ETA</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>11453001</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>XXXXXXXXXX</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
+          <t>11453001</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>XXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>Calle: calle eta mz 2 num int: lote18 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>2026-03-05T20:56:26.658Z</t>
         </is>
@@ -608,39 +638,44 @@
           <t>5555555555</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>ETA</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>11453001</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>XXXXXXXXXXXXX</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
+          <t>11453001</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>XXXXXXXXXXXXX</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>Calle: calle eta mz 1 num int: lt 2 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>2026-03-05T20:57:40.937Z</t>
         </is>
@@ -684,37 +719,62 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>consueloenmes@gmail.com</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076555958-28bsx_1.jpg</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076555958-28bsx_2.jpg</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Morelos</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>12 - 9</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>11453047</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
         <is>
           <t>Lhdi6doyf7</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>19.389539,-99.195183</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Calle: morelos 12 num int: 9 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>2026-03-09T17:15:55.959Z</t>
         </is>
@@ -758,37 +818,62 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>delvallepau@hotmail.com</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076708181-luodg_1.jpg</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076708181-luodg_2.jpg</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Etta</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>11453005</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
         <is>
           <t>Kasodjdnd</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>19.389562,-99.195197</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Calle: ETTA 6 num int: no tiene Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>2026-03-09T17:18:28.181Z</t>
         </is>
@@ -832,41 +917,66 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>emelia.hernandez@gmail.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773076721792-fhb42_1.jpg</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773076721792-fhb42_2.jpg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Eta</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
         <is>
           <t>11453001</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Emhg230578mdfrnsoo</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>19.389592,-99.195213</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Calle: calle eta mz 1 num int: lt 2 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>2026-03-09T17:18:41.808Z</t>
         </is>
@@ -910,37 +1020,62 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>lulu50@gmail.com</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076886443-evkzq_1.jpg</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773076886443-evkzq_2.jpg</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>Etta</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
         <is>
           <t>11453005</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Sosjdidkmflfll</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>19.389573,-99.195197</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Calle: Etta mz. 2 num int: lote 3 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>2026-03-09T17:22:41.521Z</t>
         </is>
@@ -984,41 +1119,66 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>mariablassil@gmail.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773076963536-avvic_1.jpg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773076963536-avvic_2.jpg</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Principal</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>10385023</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Int. 1</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Mahtmdf271198hsrn05</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>19.389588,-99.195220</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Calle: principal  8 num int: 1 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>2026-03-09T17:22:43.569Z</t>
         </is>
@@ -1062,37 +1222,62 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>malugo@aol.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077122877-ihvud_1.jpg</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077122877-ihvud_2.jpg</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Andador 2</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>10385023</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
         <is>
           <t>KHDIYDOYFIYZITZIT</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>19.389546,-99.195200</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Calle: andador 2  4 num int:  Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>2026-03-09T17:25:22.878Z</t>
         </is>
@@ -1136,41 +1321,66 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>alirile@gmail.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077186211-w4ool_1.jpg</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077186211-w4ool_2.jpg</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Capa</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>11453001</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Int. 3</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
         <is>
           <t>Rila230467mhgsrb07</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>19.389594,-99.195209</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Calle: calle capa 3 num int: 3 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>2026-03-09T17:26:26.223Z</t>
         </is>
@@ -1214,37 +1424,62 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>marcast@outlook.com</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077281530-13zzd_1.jpg</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077281530-13zzd_2.jpg</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Morelos 6A</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>11453047</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
         <is>
           <t>IGC96G96GUPGUP</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>19.389559,-99.195191</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Calle: calle  morelos  6A num int: 28 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>2026-03-09T17:28:01.530Z</t>
         </is>
@@ -1288,41 +1523,66 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>mari.lema@gmail.com</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077369199-irztr_1.jpg</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077369199-irztr_2.jpg</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>Eta</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
         <is>
           <t>11453001</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Int. 18</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Lehm431020HHGRRR15</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>19.389592,-99.195223</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Calle: calle eta mz 2 num int: lote18 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>2026-03-09T17:29:29.213Z</t>
         </is>
@@ -1366,41 +1626,66 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
+          <t>malenu@gmail.com</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077506448-35or9_1.jpg</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773077506448-35or9_2.jpg</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>Omicron</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
         <is>
           <t>11453024</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>Numl120789mdfgrsn01</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>19.389574,-99.195211</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Calle: OMICRON MZ6 num int: LT10 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>2026-03-09T17:31:46.488Z</t>
         </is>
@@ -1444,37 +1729,62 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
+          <t>sanchezcris@gmail.com</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077818445-o9t3x_1.jpg</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077818445-o9t3x_2.jpg</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>Omicron</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>2 - 2</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>11453024</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
         <is>
           <t>JADIGLGLSMSK</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>19.389574,-99.195189</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Calle: omicron 2 num int: 2 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>2026-03-09T17:36:58.445Z</t>
         </is>
@@ -1518,37 +1828,62 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
+          <t>luciestmart@hotmail.com</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077939013-u8kge_1.jpg</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>fotos/ines_pacheco/device-z9p72n/1773077939013-u8kge_2.jpg</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>Antigua via la venta</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>71</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>11453047</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
         <is>
           <t>JAQKJQIWBSIHI</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="S15" t="inlineStr">
         <is>
           <t>19.389554,-99.195185</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Calle: antigua vía laventa 71 num int: 0 Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>2026-03-09T17:38:59.014Z</t>
         </is>
@@ -1592,33 +1927,58 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>demmihy@gmail.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773078212848-kpdln_1.jpg</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773078212848-kpdln_2.jpg</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>Cda. Tehuatepec</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Maum650918mhgrt00</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>19.389574,-99.195209</t>
-        </is>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Maum650918mhgrt00</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>19.389574,-99.195209</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
         <is>
           <t>2026-03-09T17:43:32.892Z</t>
         </is>
@@ -1662,41 +2022,66 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
+          <t>gaboga45@gmail.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773078376023-8v971_1.jpg</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>fotos/maria_de_los_angeles_basurto/device-kv02so/1773078376023-8v971_2.jpg</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>Eta</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
         <is>
           <t>11453001</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>Bogg831203mdfhgrbm07</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>19.389585,-99.195207</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>Calle: calle eta me 1 lote 9 num int:  Col: Lomas de Becerra S1</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>2026-03-09T17:46:16.066Z</t>
         </is>

</xml_diff>